<commit_message>
Going for a full ANOVA based approach for the table
</commit_message>
<xml_diff>
--- a/Data/seasonal_total_CH4.xlsx
+++ b/Data/seasonal_total_CH4.xlsx
@@ -357,7 +357,7 @@
     <row r="1" s="1" customFormat="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>plot_number</t>
+          <t>Plot</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -413,7 +413,7 @@
         </is>
       </c>
       <c r="B2">
-        <v>6108.484328333199</v>
+        <v>6017.773954807674</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -426,7 +426,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>6.1084843283332</v>
+        <v>6.017773954807674</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -461,7 +461,7 @@
         </is>
       </c>
       <c r="B3">
-        <v>7097.905289484011</v>
+        <v>8741.362764658852</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -474,7 +474,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>7.097905289484011</v>
+        <v>8.741362764658852</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -509,7 +509,7 @@
         </is>
       </c>
       <c r="B4">
-        <v>1036.324843317788</v>
+        <v>-2173.915770971401</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -522,7 +522,7 @@
         </is>
       </c>
       <c r="E4">
-        <v>1.036324843317789</v>
+        <v>-2.173915770971401</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -557,7 +557,7 @@
         </is>
       </c>
       <c r="B5">
-        <v>13897.76970364108</v>
+        <v>19646.02964932226</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -570,7 +570,7 @@
         </is>
       </c>
       <c r="E5">
-        <v>13.89776970364108</v>
+        <v>19.64602964932226</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B6">
-        <v>13096.277985759</v>
+        <v>18289.76481119149</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -618,7 +618,7 @@
         </is>
       </c>
       <c r="E6">
-        <v>13.096277985759</v>
+        <v>18.28976481119149</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -653,7 +653,7 @@
         </is>
       </c>
       <c r="B7">
-        <v>12058.51230715568</v>
+        <v>15881.58215062515</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -666,7 +666,7 @@
         </is>
       </c>
       <c r="E7">
-        <v>12.05851230715568</v>
+        <v>15.88158215062515</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -701,7 +701,7 @@
         </is>
       </c>
       <c r="B8">
-        <v>1882.285316741902</v>
+        <v>1755.473902402628</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -714,7 +714,7 @@
         </is>
       </c>
       <c r="E8">
-        <v>1.882285316741902</v>
+        <v>1.755473902402628</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -749,7 +749,7 @@
         </is>
       </c>
       <c r="B9">
-        <v>3824.768839513676</v>
+        <v>3747.807221458097</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -762,7 +762,7 @@
         </is>
       </c>
       <c r="E9">
-        <v>3.824768839513676</v>
+        <v>3.747807221458097</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -797,7 +797,7 @@
         </is>
       </c>
       <c r="B10">
-        <v>2479.575645969357</v>
+        <v>2243.807197468151</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -810,7 +810,7 @@
         </is>
       </c>
       <c r="E10">
-        <v>2.479575645969357</v>
+        <v>2.243807197468151</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -845,7 +845,7 @@
         </is>
       </c>
       <c r="B11">
-        <v>5757.232404912199</v>
+        <v>7387.039866334954</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -858,7 +858,7 @@
         </is>
       </c>
       <c r="E11">
-        <v>5.757232404912199</v>
+        <v>7.387039866334955</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -893,7 +893,7 @@
         </is>
       </c>
       <c r="B12">
-        <v>24592.40441688044</v>
+        <v>31753.75974110657</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -906,7 +906,7 @@
         </is>
       </c>
       <c r="E12">
-        <v>24.59240441688044</v>
+        <v>31.75375974110657</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -941,7 +941,7 @@
         </is>
       </c>
       <c r="B13">
-        <v>3026.15476738147</v>
+        <v>3602.395026979373</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -954,7 +954,7 @@
         </is>
       </c>
       <c r="E13">
-        <v>3.02615476738147</v>
+        <v>3.602395026979373</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -989,7 +989,7 @@
         </is>
       </c>
       <c r="B14">
-        <v>1115.260972503658</v>
+        <v>1524.823611268812</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -1002,7 +1002,7 @@
         </is>
       </c>
       <c r="E14">
-        <v>1.115260972503658</v>
+        <v>1.524823611268812</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -1037,7 +1037,7 @@
         </is>
       </c>
       <c r="B15">
-        <v>3423.104665393875</v>
+        <v>3796.235398118265</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -1050,7 +1050,7 @@
         </is>
       </c>
       <c r="E15">
-        <v>3.423104665393875</v>
+        <v>3.796235398118265</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
@@ -1085,7 +1085,7 @@
         </is>
       </c>
       <c r="B16">
-        <v>5896.023325603801</v>
+        <v>6912.699865118944</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -1098,7 +1098,7 @@
         </is>
       </c>
       <c r="E16">
-        <v>5.896023325603801</v>
+        <v>6.912699865118944</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>

</xml_diff>